<commit_message>
refactor: restructure test framework and enhance module generation
- Removed global setup for authentication in Playwright tests.
- Introduced a new orchestrator for billing module tests.
- Updated email orchestrator to utilize flow resolver for better flow handling.
- Enhanced Excel to JSON conversion tool to validate flow codes and improve error handling.
- Added flow registry generation tool to automate flow imports.
- Created module generation tool to scaffold new test modules with necessary files.
- Implemented data preparation and validation tools for framework consistency.
- Added reset framework tool to clean up project artifacts with optional dry run.
- Improved test control script to dynamically find orchestrator files and handle module execution.
</commit_message>
<xml_diff>
--- a/playwright poc/data/excel/tests/Auth_Test_Cases.xlsx
+++ b/playwright poc/data/excel/tests/Auth_Test_Cases.xlsx
@@ -49,7 +49,7 @@
     <t>Expected data</t>
   </si>
   <si>
-    <t>flowKey</t>
+    <t>flowCode</t>
   </si>
   <si>
     <t>TC-AUTH-LOGIN-TC01</t>
@@ -519,18 +519,18 @@
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="27.005" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="2" width="77.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="2" width="54.29071428571429" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="2" width="19.719285714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">

</xml_diff>

<commit_message>
Refactor UsersPage locators and methods for improved readability and maintainability; update test case descriptions and configurations
</commit_message>
<xml_diff>
--- a/playwright poc/data/excel/tests/Auth_Test_Cases.xlsx
+++ b/playwright poc/data/excel/tests/Auth_Test_Cases.xlsx
@@ -571,7 +571,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="57">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="57.75">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -609,7 +609,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="82.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="84">
       <c r="A3" s="1" t="s">
         <v>23</v>
       </c>
@@ -647,7 +647,7 @@
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="82.5">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="84">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
@@ -685,7 +685,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="44.25">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="45">
       <c r="A5" s="1" t="s">
         <v>40</v>
       </c>

</xml_diff>